<commit_message>
Actualizar catálogo de minerales (M-055 Yacimiento)
</commit_message>
<xml_diff>
--- a/Coleccion de minerales.xlsx
+++ b/Coleccion de minerales.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Pascual\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Colección Minerales\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B0D9AF9-33F8-4D0F-A027-51D18613CF87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9196FD7-52B0-4B57-A21C-DC262723D6F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1265" uniqueCount="540">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1265" uniqueCount="541">
   <si>
     <t>Mineral</t>
   </si>
@@ -1756,6 +1756,9 @@
   </si>
   <si>
     <t>Matriz de roca con incrustaciones de Libethenita que aparecen como pequeños cristales verdes más oscuros y vítreos. Agregados botroidales (en forma de racimo de uvas) de Malaquita. Los nódulos presentan un color verde oscuro profundo y un brillo sedoso a aterciopelado. Conjunto bien equilibrado sobre matriz, con un crecimiento natural muy estético.</t>
+  </si>
+  <si>
+    <t>Taouz, Er Rachidia Province, Drâa-Tafilalet Region.</t>
   </si>
 </sst>
 </file>
@@ -5892,7 +5895,7 @@
         <v>375</v>
       </c>
       <c r="P56" t="s">
-        <v>333</v>
+        <v>540</v>
       </c>
       <c r="Q56" t="s">
         <v>21</v>

</xml_diff>

<commit_message>
Actualizar ficha M-015 y etiquetas del Grid (Yacimiento y Pais)
</commit_message>
<xml_diff>
--- a/Coleccion de minerales.xlsx
+++ b/Coleccion de minerales.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Colección Minerales\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9196FD7-52B0-4B57-A21C-DC262723D6F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0128076E-E918-40A2-B6EC-9F7251B90666}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1265" uniqueCount="541">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1268" uniqueCount="542">
   <si>
     <t>Mineral</t>
   </si>
@@ -1760,12 +1760,36 @@
   <si>
     <t>Taouz, Er Rachidia Province, Drâa-Tafilalet Region.</t>
   </si>
+  <si>
+    <r>
+      <t>FeO(OH)·nH</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="subscript"/>
+        <sz val="11"/>
+        <color rgb="FF202122"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF202122"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>O</t>
+    </r>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1791,6 +1815,19 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Roboto"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF202122"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <vertAlign val="subscript"/>
+      <sz val="11"/>
+      <color rgb="FF202122"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -3188,7 +3225,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:26" ht="18.75" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>283</v>
       </c>
@@ -3198,11 +3235,20 @@
       <c r="C16" t="s">
         <v>433</v>
       </c>
+      <c r="E16" t="s">
+        <v>541</v>
+      </c>
       <c r="F16" t="s">
         <v>420</v>
       </c>
+      <c r="G16" t="s">
+        <v>400</v>
+      </c>
       <c r="I16" t="s">
         <v>421</v>
+      </c>
+      <c r="K16" t="s">
+        <v>388</v>
       </c>
       <c r="L16" t="s">
         <v>351</v>

</xml_diff>

<commit_message>
Actualizar datos del excel a JSON y añadir nuevas imagenes
</commit_message>
<xml_diff>
--- a/Coleccion de minerales.xlsx
+++ b/Coleccion de minerales.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Mi Colección de Minerales\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Colección Minerales\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C5C977D-9FD8-452F-A55E-4761129B7E70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{058A903D-CF89-41A7-81CC-A119283C3027}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1334" uniqueCount="570">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1353" uniqueCount="575">
   <si>
     <t>Mineral</t>
   </si>
@@ -1865,6 +1865,21 @@
   </si>
   <si>
     <t>Mineral principal: Galena (cristales cúbicos, gris plomo, alto brillo metálico). Asociación: Pirita bien cristalizada (micro a pequeños cubos dorados). Presentación: pieza “escultural”, vertical.</t>
+  </si>
+  <si>
+    <t>M-072</t>
+  </si>
+  <si>
+    <t>590x300x440</t>
+  </si>
+  <si>
+    <t>Pentagonodecaédrico</t>
+  </si>
+  <si>
+    <t>Octaédrico</t>
+  </si>
+  <si>
+    <t>Agrupación compacta de cristales cúbicos y octaédricos, con desarrollo escalonado y fuerte predominio de caras bien definidas. Presenta brillo metálico muy intenso y color amarillo latón profundo, característico de la pirita de Huanzala. Las superficies muestran excelente reflectividad, con aristas nítidas y hábitos cristalinos robustos. Se observan leves contactos y pequeñas imperfecciones menores propias del crecimiento en matriz, sin comprometer la calidad estética global del conjunto.</t>
   </si>
 </sst>
 </file>
@@ -2318,7 +2333,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Z72"/>
+  <dimension ref="A1:Z73"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.28515625" bestFit="1" customWidth="1"/>
@@ -2331,7 +2346,7 @@
     <col min="9" max="10" width="13.140625" customWidth="1"/>
     <col min="11" max="11" width="37.140625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="16.28515625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="19.140625" customWidth="1"/>
     <col min="14" max="14" width="10.5703125" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="44.85546875" customWidth="1"/>
     <col min="17" max="17" width="11.28515625" bestFit="1" customWidth="1"/>
@@ -2829,7 +2844,7 @@
         <v>345</v>
       </c>
       <c r="F8" t="s">
-        <v>301</v>
+        <v>572</v>
       </c>
       <c r="G8" t="s">
         <v>346</v>
@@ -7286,6 +7301,80 @@
         <v>46071</v>
       </c>
       <c r="Z72" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="73" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A73" s="2" t="s">
+        <v>570</v>
+      </c>
+      <c r="B73" t="s">
+        <v>24</v>
+      </c>
+      <c r="C73" t="s">
+        <v>374</v>
+      </c>
+      <c r="E73" t="s">
+        <v>345</v>
+      </c>
+      <c r="F73" t="s">
+        <v>573</v>
+      </c>
+      <c r="G73" t="s">
+        <v>346</v>
+      </c>
+      <c r="H73" t="s">
+        <v>347</v>
+      </c>
+      <c r="I73" t="s">
+        <v>348</v>
+      </c>
+      <c r="J73" t="s">
+        <v>305</v>
+      </c>
+      <c r="K73" t="s">
+        <v>332</v>
+      </c>
+      <c r="L73" t="s">
+        <v>296</v>
+      </c>
+      <c r="M73" t="s">
+        <v>571</v>
+      </c>
+      <c r="O73">
+        <v>138</v>
+      </c>
+      <c r="P73" t="s">
+        <v>212</v>
+      </c>
+      <c r="Q73" t="s">
+        <v>28</v>
+      </c>
+      <c r="R73" t="s">
+        <v>300</v>
+      </c>
+      <c r="S73" t="s">
+        <v>373</v>
+      </c>
+      <c r="T73" s="6">
+        <v>46133</v>
+      </c>
+      <c r="U73">
+        <v>40</v>
+      </c>
+      <c r="V73" t="s">
+        <v>574</v>
+      </c>
+      <c r="W73" t="s">
+        <v>458</v>
+      </c>
+      <c r="X73">
+        <v>100</v>
+      </c>
+      <c r="Y73" s="6">
+        <v>46133</v>
+      </c>
+      <c r="Z73" t="s">
         <v>12</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Corregir dimensiones ficha M-072
</commit_message>
<xml_diff>
--- a/Coleccion de minerales.xlsx
+++ b/Coleccion de minerales.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Colección Minerales\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{058A903D-CF89-41A7-81CC-A119283C3027}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCDC0287-D640-4AA6-A656-EA82535B2BB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1870,9 +1870,6 @@
     <t>M-072</t>
   </si>
   <si>
-    <t>590x300x440</t>
-  </si>
-  <si>
     <t>Pentagonodecaédrico</t>
   </si>
   <si>
@@ -1880,6 +1877,9 @@
   </si>
   <si>
     <t>Agrupación compacta de cristales cúbicos y octaédricos, con desarrollo escalonado y fuerte predominio de caras bien definidas. Presenta brillo metálico muy intenso y color amarillo latón profundo, característico de la pirita de Huanzala. Las superficies muestran excelente reflectividad, con aristas nítidas y hábitos cristalinos robustos. Se observan leves contactos y pequeñas imperfecciones menores propias del crecimiento en matriz, sin comprometer la calidad estética global del conjunto.</t>
+  </si>
+  <si>
+    <t>59x30x44</t>
   </si>
 </sst>
 </file>
@@ -2844,7 +2844,7 @@
         <v>345</v>
       </c>
       <c r="F8" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="G8" t="s">
         <v>346</v>
@@ -7318,7 +7318,7 @@
         <v>345</v>
       </c>
       <c r="F73" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="G73" t="s">
         <v>346</v>
@@ -7339,7 +7339,7 @@
         <v>296</v>
       </c>
       <c r="M73" t="s">
-        <v>571</v>
+        <v>574</v>
       </c>
       <c r="O73">
         <v>138</v>
@@ -7363,7 +7363,7 @@
         <v>40</v>
       </c>
       <c r="V73" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="W73" t="s">
         <v>458</v>

</xml_diff>